<commit_message>
feat(import): validate asset code and serial identity on bulk import
V1-D: parity validation import asset với create/edit (ADR-IMM00-ASSETCODE).

- services/import_validators.py: AssetImportValidator kiểm tra asset_code
  pattern (chữ/số + . _ - /, no whitespace), reserved-prefix, và duplicate
  manufacturer_sn theo lô.
- utils/import_helpers.py: export_labels VI cho cột mã/serial.
- docs/res/imports/generate_templates.py + 03_danh_sach_tai_san.xlsx: regen
  template tách cột Mã tài sản ↔ Số serial NSX.
- views/asset/AssetListView.vue: IMPORT_NOTICE phân biệt rõ Mã tài sản vs
  Số serial NSX (chỉ phần ghi chú import).
- tests/test_import_asset_identity.py: phủ pattern/reserved/dup-serial +
  TestQrGenCoverageImport.
</commit_message>
<xml_diff>
--- a/assetcore/public/import_templates/03_danh_sach_tai_san.xlsx
+++ b/assetcore/public/import_templates/03_danh_sach_tai_san.xlsx
@@ -717,7 +717,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Mã tài sản (nội bộ)</t>
+          <t>Mã tài sản</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Số serial (NSX)</t>
+          <t>Số serial NSX</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Mã quản lý nội bộ duy nhất. Để trống = tự sinh.</t>
+          <t>Mã định danh nội bộ duy nhất. Chỉ chữ, số và . _ - / (không khoảng trắng, không dấu). Để trống = hệ thống tự sinh.</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Số serial do nhà sản xuất cấp (Serial Number).</t>
+          <t>Số serial do nhà sản xuất cấp — KHÁC Mã tài sản. Không bắt buộc; nếu nhập phải duy nhất.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">

</xml_diff>